<commit_message>
ready for multiple arduino style boards
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Electronics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Vehicle Connector" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Paddle Switch Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Paddle Sensor Detail" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Arduino Libraries" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Pin Reference" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -686,7 +686,7 @@
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Last Verified: 2026-03-20  |  Source: ArduinoCode/SYSTEM.md and .agents/skills/hardware-bom/SKILL.md</t>
+          <t>Last Verified: 2026-08-17  |  Source: ArduinoCode/SYSTEM.md and .agents/skills/hardware-bom/SKILL.md</t>
         </is>
       </c>
     </row>
@@ -733,12 +733,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Arduino Mega 2560</t>
+          <t>Arduino Uno (default), Mega 2560, or Nano</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ATmega2560 MCU, 54 digital I/O, 16 analog, 5V logic, 256KB flash</t>
+          <t>5V Arduino board supported by current firmware; same project pin numbers on either board</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Original or compatible clone. Do NOT use Uno — insufficient I/O pins and flash memory.</t>
+          <t>Original or compatible clone. Display DIN/CLK use each board's fixed hardware SPI pins automatically.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -873,17 +873,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Paddle Switch</t>
+          <t>Paddle Trigger Sensor</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Omron D2JW-01K11, SPDT N/O momentary, straight lever, IP67, 30VDC/100mA, chassis mount</t>
+          <t>IR slot-type optocoupler module, LM393-based, 3.3V–5V, VCC/GND/DO, digital output only</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Omron D2JW-01K11</t>
+          <t>Generic / unbranded</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>IP67 waterproof. 100,000 electrical cycle life. NOT interchangeable with D2F-5L (pocket depth differs by 1.6 mm).</t>
+          <t>Current intended build. Caveats only: generic/unbranded part, supplier stock unverified, bare PCB needs protection, rigid mounting, and strain relief.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Unverified sourcing — build intent confirmed</t>
         </is>
       </c>
     </row>
@@ -1279,32 +1279,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="17" t="inlineStr">
         <is>
-          <t>Paddle Switch — Omron D2JW-01K11</t>
+          <t>Paddle Trigger Sensor — IR Slot-Type Optocoupler (LM393-based)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Selected switch for HappyPaddleShifterCo paddle hardware</t>
+          <t>Current intended paddle input design for HappyPaddleShifterCo</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Source: Omron D2JW-01K11 datasheet, verified 2026-03-20</t>
+          <t>Source: .agents/skills/hardware-bom/SKILL.md, Models/README.md, ArduinoCode/SYSTEM.md — verified 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1328,11 +1328,11 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>ELECTRICAL SPECIFICATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
+          <t>CONFIRMED ELECTRICAL FACTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1340,16 +1340,16 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Contact Configuration</t>
+          <t>Sensor type</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SPDT (normally-open + normally-closed contacts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
+          <t>Confirmed — slot-type IR optocoupler / photointerrupter, not Hall effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
       <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1357,16 +1357,16 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>Voltage Rating</t>
+          <t>Comparator IC</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
         <is>
-          <t>30 VDC</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
+          <t>Confirmed — LM393</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1374,16 +1374,16 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Current Rating</t>
+          <t>Operating voltage</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>100 mA DC</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
+          <t>Confirmed — 3.3V to 5V, compatible with Uno, Mega, or Nano logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
       <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1391,16 +1391,16 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Operating Force</t>
+          <t>Pins</t>
         </is>
       </c>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>82 gf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
+          <t>Confirmed — VCC, GND, DO (digital output only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1408,16 +1408,16 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Release Force</t>
+          <t>Output type</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>16 gf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
+          <t>Confirmed — actively driven push-pull; Arduino input must be plain INPUT, not INPUT_PULLUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
       <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1425,16 +1425,16 @@
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>Electrical Life</t>
+          <t>Output polarity</t>
         </is>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
-          <t>100,000 cycles (~13.7 years at 20 shifts/day)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
+          <t>Confirmed — slot unobstructed = DO LOW; slot obstructed = DO HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1442,16 +1442,16 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Mechanical Life</t>
+          <t>At-rest orientation</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>1,000,000 cycles</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
+          <t>Confirmed — tab sits in the slot at rest, so DO is HIGH at rest; paddle pull clears the slot and drives DO LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
       <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1459,16 +1459,16 @@
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>Operating Temperature</t>
+          <t>Trigger edge used by firmware</t>
         </is>
       </c>
       <c r="C13" s="22" t="inlineStr">
         <is>
-          <t>−40°C to +85°C</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
+          <t>Confirmed — same HIGH→LOW falling edge as the previous logic expected</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Electrical</t>
@@ -1476,248 +1476,180 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>IP Rating</t>
+          <t>IP / environmental rating</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>IP67 — dust-tight and fully waterproof</t>
+          <t>Confirmed limitation — none stated; module ships as a bare PCB</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>MECHANICAL / MOUNTING</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
+          <t>CURRENT BUILD CAVEATS / MITIGATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>Build status</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Part sourcing</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Unverified — generic/unbranded module, no stable manufacturer part number; verify supplier stock before relying on repeat availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Build status</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>PCB protection</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed requirement — protect the bare PCB against vibration and moisture (for example conformal coat or potting after validation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Build status</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Wire termination</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed requirement — solder leads directly to the board; skip vibration-sensitive plug-in connectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Build status</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Strain relief</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Confirmed requirement — add strain relief at the sensor PCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Build status</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Mounting method</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed requirement — rigid-mount the sensor board to the paddle body; do not leave it free-hanging</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
           <t>Mechanical</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Actuator Type</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Lever, Straight</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>PCB dimensions</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>Pending research — exact module length, width, and thickness not yet confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Mechanical</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
-        <is>
-          <t>Body Width</t>
-        </is>
-      </c>
-      <c r="C17" s="22" t="inlineStr">
-        <is>
-          <t>12.7 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Slot gap dimensions</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Pending research — do not assume slot width or depth until sourced or measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Mechanical</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Body Height</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>12.3 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Mounting hole layout</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>Pending research — hole presence, positions, and diameters not yet confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Mechanical</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>Body Depth</t>
-        </is>
-      </c>
-      <c r="C19" s="22" t="inlineStr">
-        <is>
-          <t>5.3 mm ± 0.1 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Mounting Hole Diameter</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>2.35 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B21" s="22" t="inlineStr">
-        <is>
-          <t>Mounting Hole Spacing</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>3.95 × 3.95 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Lever Arc Radius</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>R16.5 mm (stainless steel t0.3 mm)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>Operating Position (lever tip travel)</t>
-        </is>
-      </c>
-      <c r="C23" s="22" t="inlineStr">
-        <is>
-          <t>8.4 mm ± 0.8 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Pretravel</t>
+          <t>Mounting fastener spec</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>6.4 mm max</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="22" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B25" s="22" t="inlineStr">
-        <is>
-          <t>Overtravel</t>
-        </is>
-      </c>
-      <c r="C25" s="22" t="inlineStr">
-        <is>
-          <t>1.4 mm min</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Movement Differential</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>0.7 mm max</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="22" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B27" s="22" t="inlineStr">
-        <is>
-          <t>Termination</t>
-        </is>
-      </c>
-      <c r="C27" s="22" t="inlineStr">
-        <is>
-          <t>Solder lug — short wire leads to PCB/Arduino</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Mechanical</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Mount Type</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Chassis mount — screws directly to 3D-printed paddle body</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="8" customHeight="1"/>
-    <row r="30" ht="50" customHeight="1">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t>3D PRINT NOTE: Switch pocket must place lever tip 8.4 mm from paddle contact surface. This is 1.6 mm DEEPER than the former D2F-5L pocket (6.8 mm). The D2JW-01K11 and D2F-5L are NOT dimensionally interchangeable.</t>
+          <t>Pending research — depends on the not-yet-confirmed module geometry and paddle pocket design</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="8" customHeight="1"/>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>INTEGRATION NOTE: This sensor needs a slot-type paddle geometry, not a lever-switch pocket. Mechanical pocket dimensions remain Pending research until the module is sourced or measured.</t>
         </is>
       </c>
     </row>
@@ -1726,8 +1658,8 @@
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A30:C30"/>
     <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1848,7 +1780,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Hardware SPI. On Mega 2560: pin 51 = MOSI (DIN), pin 52 = SCK (CLK). These pins are FIXED and cannot be reassigned.</t>
+          <t>Hardware SPI. Uno uses MOSI 11 / SCK 13; Mega uses MOSI 51 / SCK 52. DIN/CLK are fixed per board and selected automatically by the SPI library.</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1814,7 @@
     <row r="1">
       <c r="A1" s="27" t="inlineStr">
         <is>
-          <t>Arduino Mega 2560 — Pin Assignments</t>
+          <t>Arduino Uno (default) / Mega 2560 / Nano — Pin Assignments</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1828,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>WARNING: Solenoid pins (11, 12, 13) must connect via relay/driver board ONLY — never directly.</t>
+          <t>WARNING: Solenoid outputs A0, A1, and A2 must connect via relay/driver board ONLY. Display DIN/CLK stay on each board's fixed hardware SPI pins.</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1877,12 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>INPUT_PULLUP</t>
+          <t>INPUT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Shift Up paddle → GND</t>
+          <t>Shift Up paddle sensor DO</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1960,7 +1892,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Active LOW. Triggers on falling edge. 50ms debounce.</t>
+          <t>Sensor drives the line. Tab sits in slot at rest = HIGH; pull clears slot = LOW. Falling-edge trigger, 50ms debounce.</t>
         </is>
       </c>
     </row>
@@ -1977,12 +1909,12 @@
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>INPUT_PULLUP</t>
+          <t>INPUT</t>
         </is>
       </c>
       <c r="D6" s="30" t="inlineStr">
         <is>
-          <t>Shift Down paddle → GND</t>
+          <t>Shift Down paddle sensor DO</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
@@ -1992,7 +1924,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Active LOW. Triggers on falling edge. 50ms debounce.</t>
+          <t>Sensor drives the line. Tab sits in slot at rest = HIGH; pull clears slot = LOW. Falling-edge trigger, 50ms debounce.</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2059,7 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>A0</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -2159,7 +2091,7 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -2191,7 +2123,7 @@
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -2223,7 +2155,7 @@
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>11 (Uno) / 51 (Mega)</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -2248,14 +2180,14 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Fixed hardware SPI MOSI on Mega 2560. Cannot be reassigned to another pin.</t>
+          <t>Fixed hardware SPI MOSI. Board-specific, cannot be reassigned, and selected automatically by the SPI library.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>13 (Uno) / 52 (Mega)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -2280,7 +2212,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Fixed hardware SPI SCK on Mega 2560. Cannot be reassigned to another pin.</t>
+          <t>Fixed hardware SPI SCK. Board-specific, cannot be reassigned, and selected automatically by the SPI library.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
rename ArduinoCode/ to Firmware/ and knowledge/arduino/ to knowledge/microcontroller/
Multi-controller-pivot chunk 02: both folder names were vendor-scoped
(Arduino-specific) even though most content underneath was already
board-agnostic. Renamed via git mv to preserve history; target names
confirmed by human operator. Updated every live reference across the
repo; historical HANDOFFS.md/DECISIONS.md entries and the pivot chunk
prompt files were left referencing the old names deliberately, since
they're accurate records of what those names were at the time.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -686,7 +686,7 @@
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Last Verified: 2026-08-17  |  Source: ArduinoCode/SYSTEM.md and .agents/skills/hardware-bom/SKILL.md</t>
+          <t>Last Verified: 2026-08-17  |  Source: Firmware/SYSTEM.md and .agents/skills/hardware-bom/SKILL.md</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Source: .agents/skills/hardware-bom/SKILL.md, Models/README.md, ArduinoCode/SYSTEM.md — verified 2026-08-17</t>
+          <t>Source: .agents/skills/hardware-bom/SKILL.md, Models/README.md, Firmware/SYSTEM.md — verified 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Source of truth: ArduinoCode/SYSTEM.md — do not modify this table independently of the firmware spec</t>
+          <t>Source of truth: Firmware/SYSTEM.md — do not modify this table independently of the firmware spec</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
We officially bench tested the shift up and shift down while in drive
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -686,7 +686,7 @@
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Last Verified: 2026-08-17  |  Source: Firmware/SYSTEM.md and .agents/skills/hardware-bom/SKILL.md</t>
+          <t>Last Verified: 2026-08-17  |  Source: Firmware/ArduinoCode/SYSTEM.md and .agents/skills/hardware-bom/SKILL.md</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Source: .agents/skills/hardware-bom/SKILL.md, Models/README.md, Firmware/SYSTEM.md — verified 2026-08-17</t>
+          <t>Source: .agents/skills/hardware-bom/SKILL.md, Models/README.md, Firmware/ArduinoCode/SYSTEM.md — verified 2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Confirmed — tab sits in the slot at rest, so DO is HIGH at rest; paddle pull clears the slot and drives DO LOW</t>
+          <t>Confirmed by multimeter on bench hardware 2026-08-20 — tab sits in the slot at rest, so DO is LOW at rest (0V); paddle pull clears the slot and drives DO HIGH (4.3V). Opposite of the original 2026-08-17 assumption.</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C13" s="22" t="inlineStr">
         <is>
-          <t>Confirmed — same HIGH→LOW falling edge as the previous logic expected</t>
+          <t>Confirmed — LOW→HIGH rising edge</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
     <row r="2">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Source of truth: Firmware/SYSTEM.md — do not modify this table independently of the firmware spec</t>
+          <t>Source of truth: Firmware/ArduinoCode/SYSTEM.md — do not modify this table independently of the firmware spec</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Sensor drives the line. Tab sits in slot at rest = HIGH; pull clears slot = LOW. Falling-edge trigger, 50ms debounce.</t>
+          <t>Sensor drives the line. Tab sits in slot at rest = LOW; pull clears slot = HIGH. Rising-edge trigger, 50ms debounce.</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Sensor drives the line. Tab sits in slot at rest = HIGH; pull clears slot = LOW. Falling-edge trigger, 50ms debounce.</t>
+          <t>Sensor drives the line. Tab sits in slot at rest = LOW; pull clears slot = HIGH. Rising-edge trigger, 50ms debounce.</t>
         </is>
       </c>
     </row>

</xml_diff>